<commit_message>
Factory: Orta/Zor/Çok zor deep run under 4-b merged (37/40 slots with >= 2 finalists; 10 and 28 have one, 34 none); decision log; Excel Fabrika sheet; the 40-slot pass-rate report runs on demand
Unity 511/512 before this change: the only failure was the pass-rate report hitting its timeout.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/analiz/Seviye_Planlama.xlsx
+++ b/docs/analiz/Seviye_Planlama.xlsx
@@ -3518,6 +3518,9 @@
       <c r="H2" t="n">
         <v>60</v>
       </c>
+      <c r="I2" t="n">
+        <v>2.22</v>
+      </c>
       <c r="J2" t="n">
         <v>1.65</v>
       </c>
@@ -3574,6 +3577,9 @@
       <c r="H3" t="n">
         <v>35</v>
       </c>
+      <c r="I3" t="n">
+        <v>2.04</v>
+      </c>
       <c r="J3" t="n">
         <v>1.62</v>
       </c>
@@ -3615,7 +3621,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>C03-f8b82813</t>
+          <t>C03-40f02903</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -3632,31 +3638,34 @@
         <v>30</v>
       </c>
       <c r="H4" t="n">
-        <v>60</v>
+        <v>65</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2.28</v>
       </c>
       <c r="J4" t="n">
-        <v>1.77</v>
+        <v>2.19</v>
       </c>
       <c r="K4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>0.986</v>
+        <v>0.984</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>0.014</v>
+        <v>0.016</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>0.986</v>
+        <v>0.984</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>0.995</v>
+        <v>0.996</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>0.024</v>
+        <v>0.026</v>
       </c>
     </row>
     <row r="5">
@@ -3671,7 +3680,7 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>C04-71a9b229</t>
+          <t>C04-047aa68d</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -3690,29 +3699,32 @@
       <c r="H5" t="n">
         <v>45</v>
       </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
       <c r="J5" t="n">
-        <v>1.46</v>
+        <v>1.86</v>
       </c>
       <c r="K5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>0.984</v>
+        <v>0.981</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>0.968</v>
+        <v>0.966</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>0.984</v>
+        <v>0.983</v>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>0.049</v>
+        <v>0.039</v>
       </c>
     </row>
     <row r="6">
@@ -3750,6 +3762,9 @@
       <c r="H6" t="n">
         <v>60</v>
       </c>
+      <c r="I6" t="n">
+        <v>2.24</v>
+      </c>
       <c r="J6" t="n">
         <v>1.83</v>
       </c>
@@ -3787,13 +3802,54 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C06-0f100185</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>5×6</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>30</v>
+      </c>
+      <c r="H7" t="n">
+        <v>55</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="J7" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="K7" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>0.954</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>0.895</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>0.966</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -3831,6 +3887,9 @@
       <c r="H8" t="n">
         <v>60</v>
       </c>
+      <c r="I8" t="n">
+        <v>2.3</v>
+      </c>
       <c r="J8" t="n">
         <v>1.7</v>
       </c>
@@ -3887,6 +3946,9 @@
       <c r="H9" t="n">
         <v>55</v>
       </c>
+      <c r="I9" t="n">
+        <v>2.1</v>
+      </c>
       <c r="J9" t="n">
         <v>1.71</v>
       </c>
@@ -3947,6 +4009,9 @@
       <c r="H10" t="n">
         <v>60</v>
       </c>
+      <c r="I10" t="n">
+        <v>2.25</v>
+      </c>
       <c r="J10" t="n">
         <v>1.8</v>
       </c>
@@ -3984,13 +4049,54 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C10-163b2367</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>6×6</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>36</v>
+      </c>
+      <c r="H11" t="n">
+        <v>50</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="J11" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="K11" t="n">
+        <v>7</v>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>0.773</v>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>0.227</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>0.8149999999999999</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>0.243</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -4024,6 +4130,9 @@
       <c r="H12" t="n">
         <v>60</v>
       </c>
+      <c r="I12" t="n">
+        <v>2.11</v>
+      </c>
       <c r="J12" t="n">
         <v>2.17</v>
       </c>
@@ -4084,6 +4193,9 @@
       <c r="H13" t="n">
         <v>55</v>
       </c>
+      <c r="I13" t="n">
+        <v>2.27</v>
+      </c>
       <c r="J13" t="n">
         <v>1.66</v>
       </c>
@@ -4121,13 +4233,54 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C13-51d0b947</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>6×6</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>34</v>
+      </c>
+      <c r="H14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="J14" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="K14" t="n">
+        <v>8</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>0.888</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>0.963</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0.73</v>
       </c>
     </row>
     <row r="15">
@@ -4142,13 +4295,54 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C14-bb52f55f</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>6×6</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>35</v>
+      </c>
+      <c r="H15" t="n">
+        <v>50</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J15" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="K15" t="n">
+        <v>7</v>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>0.641</v>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>0.826</v>
+      </c>
+      <c r="Q15" s="2" t="n">
+        <v>0.242</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.62</v>
       </c>
     </row>
     <row r="16">
@@ -4186,6 +4380,9 @@
       <c r="H16" t="n">
         <v>60</v>
       </c>
+      <c r="I16" t="n">
+        <v>2.3</v>
+      </c>
       <c r="J16" t="n">
         <v>1.67</v>
       </c>
@@ -4223,13 +4420,54 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C16-866b071d</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>6×6</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>34</v>
+      </c>
+      <c r="H17" t="n">
+        <v>60</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="J17" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="K17" t="n">
+        <v>8</v>
+      </c>
+      <c r="L17" s="2" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>0.895</v>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="Q17" s="2" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="18">
@@ -4244,13 +4482,54 @@
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C17-73ba08a9</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>6×6</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>33</v>
+      </c>
+      <c r="H18" t="n">
+        <v>50</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="J18" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="K18" t="n">
+        <v>7</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>0.781</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>0.219</v>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>0.648</v>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="Q18" s="2" t="n">
+        <v>0.204</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0.75</v>
       </c>
     </row>
     <row r="19">
@@ -4265,7 +4544,7 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C18-5d5d65ab</t>
+          <t>C18-1107bea7</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -4279,34 +4558,37 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H19" t="n">
         <v>55</v>
       </c>
+      <c r="I19" t="n">
+        <v>2.05</v>
+      </c>
       <c r="J19" t="n">
-        <v>1.6</v>
+        <v>2.02</v>
       </c>
       <c r="K19" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>0.986</v>
+        <v>0.987</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0.014</v>
+        <v>0.013</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O19" s="2" t="n">
-        <v>0.971</v>
+        <v>0.965</v>
       </c>
       <c r="P19" s="2" t="n">
-        <v>0.986</v>
+        <v>0.988</v>
       </c>
       <c r="Q19" s="2" t="n">
-        <v>0.037</v>
+        <v>0.045</v>
       </c>
     </row>
     <row r="20">
@@ -4321,13 +4603,54 @@
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C19-f6b3e601</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>6×6</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>33</v>
+      </c>
+      <c r="H20" t="n">
+        <v>50</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="J20" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="K20" t="n">
+        <v>5</v>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>0.757</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>0.243</v>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>0.841</v>
+      </c>
+      <c r="Q20" s="2" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -4365,6 +4688,9 @@
       <c r="H21" t="n">
         <v>75</v>
       </c>
+      <c r="I21" t="n">
+        <v>2.31</v>
+      </c>
       <c r="J21" t="n">
         <v>2.39</v>
       </c>
@@ -4402,7 +4728,7 @@
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>C21-99e8e569</t>
+          <t>C21-37f1c6f3</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -4412,38 +4738,41 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>5×5</t>
+          <t>5×6</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="H22" t="n">
-        <v>45</v>
+        <v>55</v>
+      </c>
+      <c r="I22" t="n">
+        <v>2.08</v>
       </c>
       <c r="J22" t="n">
-        <v>2.08</v>
+        <v>1.77</v>
       </c>
       <c r="K22" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>0.981</v>
+        <v>0.982</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>0.019</v>
+        <v>0.018</v>
       </c>
       <c r="N22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O22" s="2" t="n">
-        <v>0.963</v>
+        <v>0.965</v>
       </c>
       <c r="P22" s="2" t="n">
         <v>0.984</v>
       </c>
       <c r="Q22" s="2" t="n">
-        <v>0.044</v>
+        <v>0.043</v>
       </c>
     </row>
     <row r="23">
@@ -4458,13 +4787,54 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C22-5614b55b</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>6×6</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>33</v>
+      </c>
+      <c r="H23" t="n">
+        <v>70</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J23" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="K23" t="n">
+        <v>5</v>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>0.841</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>0.159</v>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>0.442</v>
+      </c>
+      <c r="P23" s="2" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="Q23" s="2" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0.86</v>
       </c>
     </row>
     <row r="24">
@@ -4502,6 +4872,9 @@
       <c r="H24" t="n">
         <v>45</v>
       </c>
+      <c r="I24" t="n">
+        <v>2.21</v>
+      </c>
       <c r="J24" t="n">
         <v>1.33</v>
       </c>
@@ -4539,13 +4912,54 @@
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C24-198d2289</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>6×6</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>35</v>
+      </c>
+      <c r="H25" t="n">
+        <v>65</v>
+      </c>
+      <c r="I25" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="J25" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="K25" t="n">
+        <v>8</v>
+      </c>
+      <c r="L25" s="2" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>0.897</v>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="Q25" s="2" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="26">
@@ -4560,13 +4974,54 @@
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C25-24c94cef</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>6×6</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>33</v>
+      </c>
+      <c r="H26" t="n">
+        <v>75</v>
+      </c>
+      <c r="I26" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="J26" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="K26" t="n">
+        <v>6</v>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>0.528</v>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>0.884</v>
+      </c>
+      <c r="Q26" s="2" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0.61</v>
       </c>
     </row>
     <row r="27">
@@ -4581,7 +5036,7 @@
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>C26-8cbc73d9</t>
+          <t>C26-31e86877</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -4595,34 +5050,37 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H27" t="n">
-        <v>60</v>
+        <v>55</v>
+      </c>
+      <c r="I27" t="n">
+        <v>2.07</v>
       </c>
       <c r="J27" t="n">
-        <v>1.95</v>
+        <v>1.79</v>
       </c>
       <c r="K27" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0.991</v>
+        <v>0.986</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.014</v>
       </c>
       <c r="N27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O27" s="2" t="n">
-        <v>0.95</v>
+        <v>0.971</v>
       </c>
       <c r="P27" s="2" t="n">
-        <v>0.991</v>
+        <v>0.986</v>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>0.023</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="28">
@@ -4637,13 +5095,54 @@
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C27-71616439</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>5×6</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>29</v>
+      </c>
+      <c r="H28" t="n">
+        <v>55</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="J28" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="K28" t="n">
+        <v>8</v>
+      </c>
+      <c r="L28" s="2" t="n">
+        <v>0.946</v>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="2" t="n">
+        <v>0.898</v>
+      </c>
+      <c r="P28" s="2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="R28" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -4658,13 +5157,54 @@
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C28-d58077d1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>6×6</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>33</v>
+      </c>
+      <c r="H29" t="n">
+        <v>50</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J29" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="K29" t="n">
+        <v>7</v>
+      </c>
+      <c r="L29" s="2" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="N29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="2" t="n">
+        <v>0.482</v>
+      </c>
+      <c r="P29" s="2" t="n">
+        <v>0.793</v>
+      </c>
+      <c r="Q29" s="2" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="R29" t="n">
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="30">
@@ -4679,7 +5219,7 @@
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>C29-b1c2e769</t>
+          <t>C29-2d9dcde3</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -4689,38 +5229,41 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>5×6</t>
+          <t>5×5</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H30" t="n">
-        <v>65</v>
+        <v>45</v>
+      </c>
+      <c r="I30" t="n">
+        <v>2.09</v>
       </c>
       <c r="J30" t="n">
-        <v>2.05</v>
+        <v>1.63</v>
       </c>
       <c r="K30" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>0.993</v>
+        <v>0.984</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>0.007</v>
+        <v>0.016</v>
       </c>
       <c r="N30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O30" s="2" t="n">
-        <v>0.955</v>
+        <v>0.965</v>
       </c>
       <c r="P30" s="2" t="n">
-        <v>0.993</v>
+        <v>0.984</v>
       </c>
       <c r="Q30" s="2" t="n">
-        <v>0.013</v>
+        <v>0.045</v>
       </c>
     </row>
     <row r="31">
@@ -4735,13 +5278,54 @@
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C30-37066ecb</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>6×7</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>39</v>
+      </c>
+      <c r="H31" t="n">
+        <v>60</v>
+      </c>
+      <c r="I31" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="J31" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="K31" t="n">
+        <v>6</v>
+      </c>
+      <c r="L31" s="2" t="n">
+        <v>0.671</v>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>0.329</v>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>0.706</v>
+      </c>
+      <c r="Q31" s="2" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0.78</v>
       </c>
     </row>
     <row r="32">
@@ -4756,7 +5340,7 @@
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>C31-628e9a39</t>
+          <t>C31-ee07d843</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -4766,38 +5350,41 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>5×6</t>
+          <t>4×5</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="H32" t="n">
-        <v>65</v>
+        <v>35</v>
+      </c>
+      <c r="I32" t="n">
+        <v>2.17</v>
       </c>
       <c r="J32" t="n">
-        <v>2.3</v>
+        <v>1.29</v>
       </c>
       <c r="K32" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>0.989</v>
+        <v>0.982</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>0.011</v>
+        <v>0.018</v>
       </c>
       <c r="N32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O32" s="2" t="n">
-        <v>0.955</v>
+        <v>0.967</v>
       </c>
       <c r="P32" s="2" t="n">
-        <v>0.989</v>
+        <v>0.982</v>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>0.016</v>
+        <v>0.041</v>
       </c>
     </row>
     <row r="33">
@@ -4812,13 +5399,54 @@
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C32-89d50505</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>6×6</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>34</v>
+      </c>
+      <c r="H33" t="n">
+        <v>50</v>
+      </c>
+      <c r="I33" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="J33" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="K33" t="n">
+        <v>7</v>
+      </c>
+      <c r="L33" s="2" t="n">
+        <v>0.795</v>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="P33" s="2" t="n">
+        <v>0.837</v>
+      </c>
+      <c r="Q33" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="R33" t="n">
+        <v>0.87</v>
       </c>
     </row>
     <row r="34">
@@ -4833,13 +5461,54 @@
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C33-18f6ab59</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>5×6</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>30</v>
+      </c>
+      <c r="H34" t="n">
+        <v>60</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="J34" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="K34" t="n">
+        <v>7</v>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>0.956</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>0.896</v>
+      </c>
+      <c r="P34" s="2" t="n">
+        <v>0.969</v>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0.98</v>
       </c>
     </row>
     <row r="35">
@@ -4875,7 +5544,7 @@
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>C35-5858072b</t>
+          <t>C35-9255a195</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -4885,38 +5554,41 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>5×6</t>
+          <t>5×5</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="H36" t="n">
-        <v>60</v>
+        <v>40</v>
+      </c>
+      <c r="I36" t="n">
+        <v>2.03</v>
       </c>
       <c r="J36" t="n">
-        <v>1.83</v>
+        <v>1.37</v>
       </c>
       <c r="K36" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>0.99</v>
+        <v>0.979</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>0.01</v>
+        <v>0.021</v>
       </c>
       <c r="N36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O36" s="2" t="n">
-        <v>0.948</v>
+        <v>0.965</v>
       </c>
       <c r="P36" s="2" t="n">
-        <v>0.99</v>
+        <v>0.979</v>
       </c>
       <c r="Q36" s="2" t="n">
-        <v>0.022</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="37">
@@ -4931,13 +5603,54 @@
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C36-a0e5098d</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>6×6</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>33</v>
+      </c>
+      <c r="H37" t="n">
+        <v>50</v>
+      </c>
+      <c r="I37" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J37" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="K37" t="n">
+        <v>7</v>
+      </c>
+      <c r="L37" s="2" t="n">
+        <v>0.785</v>
+      </c>
+      <c r="M37" s="2" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="N37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="2" t="n">
+        <v>0.481</v>
+      </c>
+      <c r="P37" s="2" t="n">
+        <v>0.799</v>
+      </c>
+      <c r="Q37" s="2" t="n">
+        <v>0.173</v>
+      </c>
+      <c r="R37" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -4952,13 +5665,54 @@
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C37-d882b223</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>6×6</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>36</v>
+      </c>
+      <c r="H38" t="n">
+        <v>65</v>
+      </c>
+      <c r="I38" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="J38" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="K38" t="n">
+        <v>8</v>
+      </c>
+      <c r="L38" s="2" t="n">
+        <v>0.9370000000000001</v>
+      </c>
+      <c r="M38" s="2" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="P38" s="2" t="n">
+        <v>0.951</v>
+      </c>
+      <c r="Q38" s="2" t="n">
+        <v>0.119</v>
+      </c>
+      <c r="R38" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="39">
@@ -4973,13 +5727,54 @@
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C38-2935bf97</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>6×6</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>34</v>
+      </c>
+      <c r="H39" t="n">
+        <v>65</v>
+      </c>
+      <c r="I39" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="J39" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="K39" t="n">
+        <v>7</v>
+      </c>
+      <c r="L39" s="2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="M39" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="N39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>0.483</v>
+      </c>
+      <c r="P39" s="2" t="n">
+        <v>0.801</v>
+      </c>
+      <c r="Q39" s="2" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="R39" t="n">
+        <v>0.78</v>
       </c>
     </row>
     <row r="40">
@@ -4994,7 +5789,7 @@
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>C39-d2b069fb</t>
+          <t>C39-f54076df</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -5004,38 +5799,41 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>4×5</t>
+          <t>5×5</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="H40" t="n">
-        <v>40</v>
+        <v>45</v>
+      </c>
+      <c r="I40" t="n">
+        <v>2.03</v>
       </c>
       <c r="J40" t="n">
-        <v>1.24</v>
+        <v>2.03</v>
       </c>
       <c r="K40" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>0.985</v>
+        <v>0.988</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>0.015</v>
+        <v>0.012</v>
       </c>
       <c r="N40" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O40" s="2" t="n">
-        <v>0.949</v>
+        <v>0.966</v>
       </c>
       <c r="P40" s="2" t="n">
-        <v>0.985</v>
+        <v>0.988</v>
       </c>
       <c r="Q40" s="2" t="n">
-        <v>0.013</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="41">
@@ -5050,13 +5848,54 @@
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C40-35cef61b</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>aday yok</t>
-        </is>
+          <t>finalist</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>6×7</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>38</v>
+      </c>
+      <c r="H41" t="n">
+        <v>70</v>
+      </c>
+      <c r="I41" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J41" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="K41" t="n">
+        <v>6</v>
+      </c>
+      <c r="L41" s="2" t="n">
+        <v>0.661</v>
+      </c>
+      <c r="M41" s="2" t="n">
+        <v>0.339</v>
+      </c>
+      <c r="N41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="2" t="n">
+        <v>0.299</v>
+      </c>
+      <c r="P41" s="2" t="n">
+        <v>0.674</v>
+      </c>
+      <c r="Q41" s="2" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="R41" t="n">
+        <v>0.49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>